<commit_message>
Versão com validação no próprio código e Votação Majoritária - ainda com erro
A verificação de se a resposta está correta ou não ainda falha
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -424,21 +424,368 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>AI_Model_Result</t>
+          <t>gemma-4-31b-it</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3aa6fb7a.json</t>
+          <t>44f52bb0.json</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>INCORRECT
+          <t>CORRECT
 Reasoning:
-Recuperado via Regex de Fallback.</t>
+*   Example 1:
+        Input:
+        2 0 2
+        0 2 0
+        2 0 2
+        Output: 1
+    *   Example 2:
+        Input:
+        2 0 0
+        2 0 0
+        0 2 0
+        Output: 7
+    *   Example 3:
+        Input:
+        2 0 2
+        2 0 2
+        2 0 2
+        Output: 1
+    *   Example 4:
+        Input:
+        0 0 0
+        2 0 2
+        0 0 0
+        Output: 1
+    *   Example 5:
+        Input:
+        2 2 0
+        0 2 2
+        0 0 0
+        Output: 7
+    *   Example 6:
+        Input:
+        2 2 0
+        0 2 0
+        0 0 0
+        Output: 7
+    *   All inputs are 3x3 grids.
+    *   All inputs contain only 0s and 2s.
+    *   All outputs are single-digit numbers (1 or 7).
+    *   Example 1:
+        Input:
+        2 0 2
+        0 2 0
+        2 0 2
+        Output: 1
+        Pattern: X-shaped pattern of 2s. (Diagonal 2s)
+    *   Example 2:
+        Input:
+        2 0 0
+        2 0 0
+        0 2 0
+        Output: 7
+        Pattern: Not symmetric, not a simple line.
+    *   Example 3:
+        Input:
+        2 0 2
+        2 0 2
+        2 0 2
+        Output: 1
+        Pattern: Two vertical lines of 2s. (Symmetric horizontally)
+    *   Example 4:
+        Input:
+        0 0 0
+        2 0 2
+        0 0 0
+        Output: 1
+        Pattern: One horizontal line of 2s (with a gap). (Symmetric horizontally and vertically)
+    *   Example 5:
+        Input:
+        2 2 0
+        0 2 2
+        0 0 0
+        Output: 7
+        Pattern: Not symmetric.
+    *   Example 6:
+        Input:
+        2 2 0
+        0 2 0
+        0 0 0
+        Output: 7
+        Pattern: Not symmetric.
+    *   Example 1: Symmetric (Horizontal, Vertical, Diagonal) -&gt; 1
+    *   Example 2: Not symmetric -&gt; 7
+    *   Example 3: Symmetric (Horizontal) -&gt; 1
+    *   Example 4: Symmetric (Horizontal, Vertical) -&gt; 1
+    *   Example 5: Not symmetric -&gt; 7
+    *   Example 6: Not symmetric -&gt; 7
+    Let's re-verify symmetry:
+    *   Ex 1:
+        2 0 2
+        0 2 0
+        2 0 2
+        Vertical symmetry (col 0 == col 2): Yes.
+        Horizontal symmetry (row 0 == row 2): Yes.
+        Output: 1
+    *   Ex 2:
+        2 0 0
+        2 0 0
+        0 2 0
+        Vertical symmetry (col 0 == col 2): No.
+        Horizontal symmetry (row 0 == row 2): No.
+        Output: 7
+    *   Ex 3:
+        2 0 2
+        2 0 2
+        2 0 2
+        Vertical symmetry (col 0 == col 2): Yes.
+        Horizontal symmetry (row 0 == row 2): Yes.
+        Output: 1
+    *   Ex 4:
+        0 0 0
+        2 0 2
+        0 0 0
+        Vertical symmetry (col 0 == col 2): Yes.
+        Horizontal symmetry (row 0 == row 2): Yes.
+        Output: 1
+    *   Ex 5:
+        2 2 0
+        0 2 2
+        0 0 0
+        Vertical symmetry (col 0 == col 2): No.
+        Horizontal symmetry (row 0 == row 2): No.
+        Output: 7
+    *   Ex 6:
+        2 2 0
+        0 2 0
+        0 0 0
+        Vertical symmetry (col 0 == col 2): No.
+        Horizontal symmetry (row 0 == row 2): No.
+        Output: 7
+    Wait, let's check if *any* symmetry is enough.
+    Example 1: Vertical and Horizontal symmetry.
+    Example 2: No symmetry.
+    Example 3: Vertical and Horizontal symmetry.
+    Example 4: Vertical and Horizontal symmetry.
+    Example 5: No symmetry.
+    Example 6: No symmetry.
+    Wait, is there any other pattern? Let's check the number of 2s.
+    Ex 1: five 2s -&gt; 1
+    Ex 2: three 2s -&gt; 7
+    Ex 3: six 2s -&gt; 1
+    Ex 4: two 2s -&gt; 1
+    Ex 5: four 2s -&gt; 7
+    Ex 6: three 2s -&gt; 7
+    Number of 2s doesn't seem to be the rule.
+    Let's re-examine the symmetry.
+    Ex 1: Symmetric about the vertical axis? Yes.
+    Ex 2: Symmetric about the vertical axis? No.
+    Ex 3: Symmetric about the vertical axis? Yes.
+    Ex 4: Symmetric about the vertical axis? Yes.
+    Ex 5: Symmetric about the vertical axis? No.
+    Ex 6: Symmetric about the vertical axis? No.
+    Is it just vertical symmetry?
+    Let's check:
+    Ex 1: col 0 is (2,0,2), col 2 is (2,0,2). Match.
+    Ex 2: col 0 is (2,2,0), col 2 is (0,0,0). No match.
+    Ex 3: col 0 is (2,2,2), col 2 is (2,2,2). Match.
+    Ex 4: col 0 is (0,2,0), col 2 is (0,2,0). Match.
+    Ex 5: col 0 is (2,0,0), col 2 is (0,2,0). No match.
+    Ex 6: col 0 is (2,0,0), col 2 is (0,0,0). No match.
+    Wait, let's test this rule: If the grid is vertically symmetric (col 0 == col 2), output 1. Otherwise, output 7.
+    Let's check if there are any other symmetries.
+    What about horizontal symmetry?
+    Ex 1: row 0 is (2,0,2), row 2 is (2,0,2). Match.
+    Ex 2: row 0 is (2,0,0), row 2 is (0,2,0). No match.
+    Ex 3: row 0 is (2,0,2), row 2 is (2,0,2). Match.
+    Ex 4: row 0 is (0,0,0), row 2 is (0,0,0). Match.
+    Ex 5: row 0 is (2,2,0), row 2 is (0,0,0). No match.
+    Ex 6: row 0 is (2,2,0), row 2 is (0,0,0). No match.
+    So both vertical and horizontal symmetry are present in all the "1" cases and absent in all the "7" cases.
+    Let's check the test input:
+    2 0 2
+    2 2 2
+    2 0 2
+    Vertical symmetry (col 0 == col 2):
+    col 0: (2, 2, 2)
+    col 2: (2, 2, 2)
+    Match.
+    Horizontal symmetry (row 0 == row 2):
+    row 0: (2, 0, 2)
+    row 2: (2, 0, 2)
+    Match.
+    Based on the rule (vertical symmetry or horizontal symmetry), the output should be 1.
+    Wait, let me double-check. Could there be any other rule?
+    What if it's about the center element?
+    Ex 1: center is 2 -&gt; 1
+    Ex 2: center is 0 -&gt; 7
+    Ex 3: center is 0 -&gt; 1 (Wait, Example 3 center is 0, but output is 1)
+    Ex 4: center is 0 -&gt; 1 (Example 4 center is 0, but output is 1)
+    Ex 5: center is 2 -&gt; 7 (Example 5 center is 2, but output is 7)
+    Ex 6: center is 2 -&gt; 7 (Example 6 center is 2, but output is 7)
+    So the center element is not the rule.
+    What if it's about the number of 2s in each row/column?
+    Ex 1:
+    Rows: 2, 1, 2
+    Cols: 2, 1, 2
+    Ex 2:
+    Rows: 1, 1, 1
+    Cols: 2, 0, 1
+    Ex 3:
+    Rows: 2, 2, 2
+    Cols: 3, 0, 3
+    Ex 4:
+    Rows: 0, 2, 0
+    Cols: 1, 0, 1
+    Ex 5:
+    Rows: 2, 2, 0
+    Cols: 1, 2, 1
+    Ex 6:
+    Rows: 2, 1, 0
+    Cols: 1, 2, 0
+    Let's look at the symmetry again.
+    Example 1: Symmetric V and H.
+    Example 2: Not symmetric.
+    Example 3: Symmetric V and H.
+    Example 4: Symmetric V and H.
+    Example 5: Not symmetric.
+    Example 6: Not symmetric.
+    It seems very consistent. If the grid is symmetric across the vertical axis (col 0 == col 2), the output is 1. If it's not, the output is 7. (Actually, both vertical and horizontal symmetries seem to hold for all 1s).
+    Wait, let me check Example 3 again.
+    Example 3 Input:
+    2 0 2
+    2 0 2
+    2 0 2
+    Vertical symmetry: Col 0 is (2,2,2), Col 2 is (2,2,2). Yes.
+    Horizontal symmetry: Row 0 is (2,0,2), Row 2 is (2,0,2). Yes.
+    Example 4 Input:
+    0 0 0
+    2 0 2
+    0 0 0
+    Vertical symmetry: Col 0 is (0,2,0), Col 2 is (0,2,0). Yes.
+    Horizontal symmetry: Row 0 is (0,0,0), Row 2 is (0,0,0). Yes.
+    So the rule seems to be: if the grid has vertical symmetry (col 0 == col 2), the output is 1. If it doesn't, the output is 7.
+    Let's double-check Example 5 and 6.
+    Example 5:
+    2 2 0
+    0 2 2
+    0 0 0
+    Col 0: (2,0,0), Col 2: (0,2,0). No.
+    Row 0: (2,2,0), Row 2: (0,0,0). No.
+    Output: 7.
+    Example 6:
+    2 2 0
+    0 2 0
+    0 0 0
+    Col 0: (2,0,0), Col 2: (0,0,0). No.
+    Row 0: (2,2,0), Row 2: (0,0,0). No.
+    Output: 7.
+    Test Input:
+    2 0 2
+    2 2 2
+    2 0 2
+    Col 0: (2, 2, 2)
+    Col 2: (2, 2, 2)
+    Match!
+    Row 0: (2, 0, 2)
+    Row 2: (2, 0, 2)
+    Match!
+    Wait, let me think if there's any other possible rule. What about the number 1 and 7?
+    In ARC, often 1 and 7 are colors. But here they are the outputs.
+    Is there any other property?
+    What if the rule is: "If the grid is symmetric, output 1, else output 7"?
+    Symmetry can be vertical, horizontal, or rotational.
+    In all "1" cases, the grid was both vertically and horizontally symmetric.
+    In all "7" cases, it was neither.
+    Let's check the test input again:
+    2 0 2
+    2 2 2
+    2 0 2
+    It is both vertically and horizontally symmetric.
+    One more check. Could the rule be about the number of 2s?
+    Ex 1: 5 (Odd) -&gt; 1
+    Ex 2: 3 (Odd) -&gt; 7
+    Ex 3: 6 (Even) -&gt; 1
+    Ex 4: 2 (Even) -&gt; 1
+    Ex 5: 4 (Even) -&gt; 7
+    Ex 6: 3 (Odd) -&gt; 7
+    No, that doesn't work.
+    What about the sum of the 2s?
+    Ex 1: 10 -&gt; 1
+    Ex 2: 6 -&gt; 7
+    Ex 3: 12 -&gt; 1
+    Ex 4: 4 -&gt; 1
+    Ex 5: 8 -&gt; 7
+    Ex 6: 6 -&gt; 7
+    Sums: 10, 6, 12, 4, 8, 6.
+    Outputs: 1, 7, 1, 1, 7, 7.
+    Wait!
+    10 -&gt; 1
+    6 -&gt; 7
+    12 -&gt; 1
+    4 -&gt; 1
+    8 -&gt; 7
+    6 -&gt; 7
+    If the sum is a multiple of 4?
+    10: No
+    6: No
+    12: Yes
+    4: Yes
+    8: Yes
+    6: No
+    That doesn't match (10 is not a multiple of 4, but output is 1).
+    What if the sum is...
+    4: 1
+    6: 7
+    8: 7
+    10: 1
+    12: 1
+    This doesn't seem to be a simple rule.
+    Let's go back to symmetry. It's the most plausible rule.
+    If the grid is symmetric across the vertical axis, output 1.
+    If not, output 7.
+    Wait, let me check if there's any other symmetry.
+    What about diagonal symmetry?
+    Example 1:
+    2 0 2
+    0 2 0
+    2 0 2
+    Diagonal 1 (top-left to bottom-right): (2, 2, 2).
+    Diagonal 2 (top-right to bottom-left): (2, 2, 2).
+    Symmetric across both diagonals.
+    Example 2:
+    2 0 0
+    2 0 0
+    0 2 0
+    Diagonal 1: (2, 0, 0).
+    Diagonal 2: (0, 0, 0).
+    Not symmetric.
+    Example 3:
+    2 0 2
+    2 0 2
+    2 0 2
+    Diagonal 1: (2, 0, 2).
+    Diagonal 2: (2, 0, 2).
+    Not symmetric across diagonals (e.g., (0,1) is 0, (1,0) is 2).
+    Example 4:
+    0 0 0
+    2 0 2
+    0 0 0
+    Diagonal 1: (0, 0, 0).
+    Diagonal 2: (0, 0, 0).
+    Symmetric across diagonals (e.g., (1,0) is 2, (0,1) is 0 - wait, no it's not).
+    (1,0) is 2, (0,1) is 0. Not symmetric.
+    So the only symmetry that holds for all "1" cases is vertical and horizontal symmetry.
+    Let's re-verify the vertical symmetry for all examples:
+    Ex 1: Col 0 (2,0,2), Col 2 (2,0,2). Yes.
+    Ex 2: Col 0 (2,2,0), Col 2 (0,0,0). No.
+    Ex 3: Col 0 (2,2,2), Col 2 (2,2,2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: adiciona tracking the tempo
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -431,20 +431,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>44f52bb0.json</t>
+          <t>00576224.json</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>The user wants me to extract the final predicted value from the provided reasoning text.
-The reasoning text analyzes several examples of 3x3 grids containing 0s and 2s and their corresponding output values (1 or 7).
-The reasoning concludes that if a grid has vertical and horizontal symmetry, the output is 1; otherwise, it's 7.
-The test input is:
-2 0 2
-2 2 2
-2 0 2
-The reasoning determines that this test input has both vertical and horizontal symmetry.
-Therefore, the predicted output is 1.</t>
+          <t>*   Input: 2x2 grid `[[3, 2], [7, 8]]`
+    *   Pattern:
+        *   Row 1: `a b a b a b` (3 2 3 2 3 2)
+        *   Row 2: `c d c d c d` (7 8 7 8 7 8)
+        *   Row 3: `b a b a b a` (2 3 2 3 2 3)
+        *   Row 4: `d c d c d c` (8 7 8 7 8 7)
+        *   Row 5: `a b a b a b` (3 2 3 2 3 2)
+        *   Row 6: `c d c d c d` (7 8 7 8 7 8)
+    *   Final Grid:
+        3 2 3 2 3 2
+        7 8 7 8 7 8
+        2 3 2 3 2 3
+        8 7 8 7 8 7
+        3 2 3 2 3 2
+        7 8 7 8 7 8</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: adiciona tracking the precisão (taxa de acerto) da LLM na task singular
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -436,21 +436,32 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>*   Input: 2x2 grid `[[3, 2], [7, 8]]`
-    *   Pattern:
-        *   Row 1: `a b a b a b` (3 2 3 2 3 2)
-        *   Row 2: `c d c d c d` (7 8 7 8 7 8)
-        *   Row 3: `b a b a b a` (2 3 2 3 2 3)
-        *   Row 4: `d c d c d c` (8 7 8 7 8 7)
-        *   Row 5: `a b a b a b` (3 2 3 2 3 2)
-        *   Row 6: `c d c d c d` (7 8 7 8 7 8)
-    *   Final Grid:
+          <t>The user wants me to extract the final predicted grid from the provided reasoning text.
+    *   Input:
+        3 2
+        7 8
+    *   Pattern identified:
+        Row 0: A B A B A B
+        Row 1: C D C D C D
+        Row 2: B A B A B A
+        Row 3: D C D C D C
+        Row 4: A B A B A B
+        Row 5: C D C D C D
+    *   Values: A=3, B=2, C=7, D=8
+    *   Resulting Grid:
         3 2 3 2 3 2
         7 8 7 8 7 8
         2 3 2 3 2 3
         8 7 8 7 8 7
         3 2 3 2 3 2
-        7 8 7 8 7 8</t>
+        7 8 7 8 7 8
+    *   Row 0: 3 2 3 2 3 2
+    *   Row 1: 7 8 7 8 7 8
+    *   Row 2: 2 3 2 3 2 3
+    *   Row 3: 8 7 8 7 8 7
+    *   Row 4: 3 2 3 2 3 2
+    *   Row 5: 7 8 7 8 7 8
+    The output must be only the &lt;prediction&gt; tags containing the numbers.</t>
         </is>
       </c>
     </row>

</xml_diff>